<commit_message>
Updated nutrient constraints and import commands
</commit_message>
<xml_diff>
--- a/data/nutrient_constraints.xlsx
+++ b/data/nutrient_constraints.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\welcome\feed_website\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48C5FEEE-EC64-41DC-82A2-7853A49778D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497B5245-1D13-4834-955D-8F5D1F9AA639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="53">
   <si>
     <t>life_stage</t>
   </si>
@@ -175,6 +175,15 @@
   </si>
   <si>
     <t>a_phosphorus_min</t>
+  </si>
+  <si>
+    <t>broiler</t>
+  </si>
+  <si>
+    <t>b breeder</t>
+  </si>
+  <si>
+    <t>animal_type</t>
   </si>
 </sst>
 </file>
@@ -190,7 +199,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -217,12 +228,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -230,15 +241,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,8 +577,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:40" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
-        <v>27</v>
+      <c r="A1" s="4" t="s">
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -671,7 +700,7 @@
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>28</v>
@@ -793,7 +822,7 @@
     </row>
     <row r="3" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>29</v>
@@ -915,7 +944,7 @@
     </row>
     <row r="4" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>30</v>
@@ -1037,7 +1066,7 @@
     </row>
     <row r="5" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>31</v>
@@ -1159,7 +1188,7 @@
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>32</v>
@@ -1281,7 +1310,7 @@
     </row>
     <row r="7" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>33</v>
@@ -1403,7 +1432,7 @@
     </row>
     <row r="8" spans="1:40" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>34</v>
@@ -1523,9 +1552,9 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="9" spans="1:40" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:40" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>35</v>
@@ -1647,7 +1676,7 @@
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>32</v>
@@ -1769,7 +1798,7 @@
     </row>
     <row r="11" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>30</v>
@@ -1891,7 +1920,7 @@
     </row>
     <row r="12" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>26</v>
@@ -2013,7 +2042,7 @@
     </row>
     <row r="13" spans="1:40" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>36</v>

</xml_diff>